<commit_message>
Code-and-data package updated to the current draft: figure scripts 50-53 + fig_style.R and their inputs, README (structure, Figs 1-6, appendix A1-A13, steps; XGBoost/LightGBM marked as earlier check), source data renumbered (new Fig 2, AutoGluon-only BH in Table 2); 51 AutoGluon-only; tested in a package copy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flux/paper_code_data/source_data/Table2_siteyear_MAE_bootstrap.xlsx
+++ b/data/flux/paper_code_data/source_data/Table2_siteyear_MAE_bootstrap.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="26">
   <si>
     <t>note</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Table 2: change of the pooled site-year MAE when mortality is added (AutoGluon).</t>
   </si>
   <si>
-    <t>pct = % change; pct_lo/pct_hi = 95 % site-block bootstrap interval; p_perm/q = paired permutation (sites swapped), BH-corrected across the three learners.</t>
-  </si>
-  <si>
-    <t>subset: all site-years; high = High sites; yr_midhigh / yr_high = site-years whose own relative mortality exceeds the Mid / High break.</t>
+    <t>pct = % change; pct_lo/pct_hi = 95 % site-block bootstrap interval; p_perm/q = paired permutation (sites swapped), BH-corrected across the AutoGluon site-year tests.</t>
+  </si>
+  <si>
+    <t>subset: all = all site-years; midhigh / high = all years of the Mid+High / High sites; yr_midhigh / yr_high = site-years whose own relative mortality exceeds the Mid / High break.</t>
   </si>
   <si>
     <t>response</t>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>WUE</t>
+  </si>
+  <si>
+    <t>midhigh</t>
   </si>
   <si>
     <t>high</t>
@@ -462,7 +465,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1">
@@ -532,7 +535,7 @@
         <v>0.171182881711829</v>
       </c>
       <c r="K2">
-        <v>0.192765770151957</v>
+        <v>0.171182881711829</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -567,7 +570,7 @@
         <v>0.0835916408359164</v>
       </c>
       <c r="K3">
-        <v>0.123839467905061</v>
+        <v>0.101323201013232</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -602,7 +605,7 @@
         <v>0.0223977602239776</v>
       </c>
       <c r="K4">
-        <v>0.0514234290856629</v>
+        <v>0.03555200035552</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -637,7 +640,7 @@
         <v>0.002999700029997</v>
       </c>
       <c r="K5">
-        <v>0.0156506088521583</v>
+        <v>0.01090800010908</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -707,7 +710,7 @@
         <v>0.0003999600039996</v>
       </c>
       <c r="K7">
-        <v>0.005999400059994</v>
+        <v>0.005332800053328</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -742,7 +745,7 @@
         <v>0.0236976302369763</v>
       </c>
       <c r="K8">
-        <v>0.0514234290856629</v>
+        <v>0.03555200035552</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -777,7 +780,7 @@
         <v>0.023997600239976</v>
       </c>
       <c r="K9">
-        <v>0.0514234290856629</v>
+        <v>0.03555200035552</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -791,28 +794,28 @@
         <v>22</v>
       </c>
       <c r="D10">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E10">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="F10">
-        <v>-0.00122773386165283</v>
+        <v>-0.0007707274229183521</v>
       </c>
       <c r="G10">
-        <v>-2.94197075180864</v>
+        <v>-2.06028814037544</v>
       </c>
       <c r="H10">
-        <v>-8.375869844590399</v>
+        <v>-5.25039418056846</v>
       </c>
       <c r="I10">
-        <v>2.13138272699604</v>
+        <v>1.09525253577241</v>
       </c>
       <c r="J10">
-        <v>0.128287171282872</v>
+        <v>0.103689631036896</v>
       </c>
       <c r="K10">
-        <v>0.162046953199417</v>
+        <v>0.1219878012198777</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -826,28 +829,28 @@
         <v>22</v>
       </c>
       <c r="D11">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E11">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="F11">
-        <v>-0.00218117436495249</v>
+        <v>-0.00139125428838921</v>
       </c>
       <c r="G11">
-        <v>-5.25048299349444</v>
+        <v>-3.69334130316401</v>
       </c>
       <c r="H11">
-        <v>-13.1430006443466</v>
+        <v>-7.25499787567919</v>
       </c>
       <c r="I11">
-        <v>1.24909337767268</v>
+        <v>-0.071805817701489</v>
       </c>
       <c r="J11">
-        <v>0.0591940805919408</v>
+        <v>0.023997600239976</v>
       </c>
       <c r="K11">
-        <v>0.098656800986568</v>
+        <v>0.03555200035552</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -861,28 +864,28 @@
         <v>22</v>
       </c>
       <c r="D12">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E12">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="F12">
-        <v>-0.407422486981712</v>
+        <v>-0.35150318006165</v>
       </c>
       <c r="G12">
-        <v>-7.19093289074554</v>
+        <v>-6.12976587101762</v>
       </c>
       <c r="H12">
-        <v>-18.0528336887189</v>
+        <v>-10.9151964237536</v>
       </c>
       <c r="I12">
-        <v>2.87646398667019</v>
+        <v>-1.46265082042202</v>
       </c>
       <c r="J12">
-        <v>0.108889111088891</v>
+        <v>0.009099090090990899</v>
       </c>
       <c r="K12">
-        <v>0.146754555313699</v>
+        <v>0.021409623743508</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -896,28 +899,28 @@
         <v>22</v>
       </c>
       <c r="D13">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E13">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="F13">
-        <v>-0.386929315382964</v>
+        <v>-0.485195323601988</v>
       </c>
       <c r="G13">
-        <v>-7.0535023162857</v>
+        <v>-8.28300520124635</v>
       </c>
       <c r="H13">
-        <v>-17.2276326820933</v>
+        <v>-12.6023981414942</v>
       </c>
       <c r="I13">
-        <v>3.60442454025906</v>
+        <v>-3.98249083629758</v>
       </c>
       <c r="J13">
-        <v>0.118688131186881</v>
+        <v>0.0007999200079992</v>
       </c>
       <c r="K13">
-        <v>0.153686758983676</v>
+        <v>0.0063993600639936</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -931,28 +934,28 @@
         <v>22</v>
       </c>
       <c r="D14">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E14">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="F14">
-        <v>-0.691097880501684</v>
+        <v>-0.351166347256085</v>
       </c>
       <c r="G14">
-        <v>-22.6321346731244</v>
+        <v>-11.3168217363717</v>
       </c>
       <c r="H14">
-        <v>-33.5912532572929</v>
+        <v>-17.481015644899</v>
       </c>
       <c r="I14">
-        <v>-11.0593782395689</v>
+        <v>-5.08037980606321</v>
       </c>
       <c r="J14">
-        <v>0.0007999200079992</v>
+        <v>0.0003999600039996</v>
       </c>
       <c r="K14">
-        <v>0.008726400087264</v>
+        <v>0.005332800053328</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -966,28 +969,28 @@
         <v>22</v>
       </c>
       <c r="D15">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E15">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="F15">
-        <v>-0.499947499305979</v>
+        <v>-0.327016264315909</v>
       </c>
       <c r="G15">
-        <v>-17.4786290491947</v>
+        <v>-10.5302835080963</v>
       </c>
       <c r="H15">
-        <v>-30.6844457896897</v>
+        <v>-17.3196912634385</v>
       </c>
       <c r="I15">
-        <v>-2.09408633866107</v>
+        <v>-3.39598341143336</v>
       </c>
       <c r="J15">
-        <v>0.0311968803119688</v>
+        <v>0.0045995400459954</v>
       </c>
       <c r="K15">
-        <v>0.06259374062593739</v>
+        <v>0.01476775399383139</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1001,28 +1004,28 @@
         <v>22</v>
       </c>
       <c r="D16">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E16">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="F16">
-        <v>-0.0919717941041224</v>
+        <v>-0.0489410796311922</v>
       </c>
       <c r="G16">
-        <v>-10.9330213731233</v>
+        <v>-6.84773054808714</v>
       </c>
       <c r="H16">
-        <v>-17.7875005238154</v>
+        <v>-11.2744963976347</v>
       </c>
       <c r="I16">
-        <v>-4.34069631336406</v>
+        <v>-2.31010483748635</v>
       </c>
       <c r="J16">
-        <v>0.0014998500149985</v>
+        <v>0.0016998300169983</v>
       </c>
       <c r="K16">
-        <v>0.0101989801019898</v>
+        <v>0.008443600084436001</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1036,28 +1039,28 @@
         <v>22</v>
       </c>
       <c r="D17">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E17">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="F17">
-        <v>-0.123628811696748</v>
+        <v>-0.0450009480014665</v>
       </c>
       <c r="G17">
-        <v>-14.8039028862857</v>
+        <v>-6.4011798237569</v>
       </c>
       <c r="H17">
-        <v>-23.8710768148773</v>
+        <v>-11.5077326742567</v>
       </c>
       <c r="I17">
-        <v>-6.35959789070967</v>
+        <v>-1.1650061934816</v>
       </c>
       <c r="J17">
-        <v>0.0018998100189981</v>
+        <v>0.0116988301169883</v>
       </c>
       <c r="K17">
-        <v>0.0108560572514177</v>
+        <v>0.0243975602439756</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1071,28 +1074,28 @@
         <v>23</v>
       </c>
       <c r="D18">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E18">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F18">
-        <v>-0.00142513905768987</v>
+        <v>-0.00122773386165283</v>
       </c>
       <c r="G18">
-        <v>-3.90327732690893</v>
+        <v>-2.94197075180864</v>
       </c>
       <c r="H18">
-        <v>-7.73803690498597</v>
+        <v>-8.375869844590399</v>
       </c>
       <c r="I18">
-        <v>0.00775858920047114</v>
+        <v>2.13138272699604</v>
       </c>
       <c r="J18">
-        <v>0.0296970302969703</v>
+        <v>0.128287171282872</v>
       </c>
       <c r="K18">
-        <v>0.06252006378309539</v>
+        <v>0.1350391276661811</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -1106,28 +1109,28 @@
         <v>23</v>
       </c>
       <c r="D19">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E19">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F19">
-        <v>-0.00200997216469339</v>
+        <v>-0.00218117436495249</v>
       </c>
       <c r="G19">
-        <v>-5.44671551832906</v>
+        <v>-5.25048299349444</v>
       </c>
       <c r="H19">
-        <v>-9.564714776353799</v>
+        <v>-13.1430006443466</v>
       </c>
       <c r="I19">
-        <v>-1.34184929226255</v>
+        <v>1.24909337767268</v>
       </c>
       <c r="J19">
-        <v>0.0054994500549945</v>
+        <v>0.0591940805919408</v>
       </c>
       <c r="K19">
-        <v>0.0206229377062294</v>
+        <v>0.0789254407892544</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -1141,28 +1144,28 @@
         <v>23</v>
       </c>
       <c r="D20">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E20">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F20">
-        <v>-0.38718347675304</v>
+        <v>-0.407422486981712</v>
       </c>
       <c r="G20">
-        <v>-6.70973371481666</v>
+        <v>-7.19093289074554</v>
       </c>
       <c r="H20">
-        <v>-12.8480119771694</v>
+        <v>-18.0528336887189</v>
       </c>
       <c r="I20">
-        <v>-0.681260034655301</v>
+        <v>2.87646398667019</v>
       </c>
       <c r="J20">
-        <v>0.0194980501949805</v>
+        <v>0.108889111088891</v>
       </c>
       <c r="K20">
-        <v>0.04587776516466</v>
+        <v>0.1235432012354322</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1176,28 +1179,28 @@
         <v>23</v>
       </c>
       <c r="D21">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E21">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F21">
-        <v>-0.485112114343369</v>
+        <v>-0.386929315382964</v>
       </c>
       <c r="G21">
-        <v>-8.342471246999761</v>
+        <v>-7.0535023162857</v>
       </c>
       <c r="H21">
-        <v>-14.1889752040962</v>
+        <v>-17.2276326820933</v>
       </c>
       <c r="I21">
-        <v>-2.55205053892857</v>
+        <v>3.60442454025906</v>
       </c>
       <c r="J21">
-        <v>0.0047995200479952</v>
+        <v>0.118688131186881</v>
       </c>
       <c r="K21">
-        <v>0.0197399614877222</v>
+        <v>0.1283114931750065</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1211,28 +1214,28 @@
         <v>23</v>
       </c>
       <c r="D22">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E22">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F22">
-        <v>-0.41223661230812</v>
+        <v>-0.691097880501684</v>
       </c>
       <c r="G22">
-        <v>-12.5494977568365</v>
+        <v>-22.6321346731244</v>
       </c>
       <c r="H22">
-        <v>-20.0549353616032</v>
+        <v>-33.5912532572929</v>
       </c>
       <c r="I22">
-        <v>-4.86520404681452</v>
+        <v>-11.0593782395689</v>
       </c>
       <c r="J22">
-        <v>0.0016998300169983</v>
+        <v>0.0007999200079992</v>
       </c>
       <c r="K22">
-        <v>0.0101989801019898</v>
+        <v>0.0063993600639936</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -1246,28 +1249,28 @@
         <v>23</v>
       </c>
       <c r="D23">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E23">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F23">
-        <v>-0.377330413617452</v>
+        <v>-0.499947499305979</v>
       </c>
       <c r="G23">
-        <v>-11.6114789432087</v>
+        <v>-17.4786290491947</v>
       </c>
       <c r="H23">
-        <v>-19.7712949536142</v>
+        <v>-30.6844457896897</v>
       </c>
       <c r="I23">
-        <v>-2.7325181737937</v>
+        <v>-2.09408633866107</v>
       </c>
       <c r="J23">
-        <v>0.0074992500749925</v>
+        <v>0.0311968803119688</v>
       </c>
       <c r="K23">
-        <v>0.0249704759253804</v>
+        <v>0.04303017974064662</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -1281,28 +1284,28 @@
         <v>23</v>
       </c>
       <c r="D24">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E24">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F24">
-        <v>-0.0531821350745159</v>
+        <v>-0.0919717941041224</v>
       </c>
       <c r="G24">
-        <v>-7.19617057069742</v>
+        <v>-10.9330213731233</v>
       </c>
       <c r="H24">
-        <v>-12.2095432994123</v>
+        <v>-17.7875005238154</v>
       </c>
       <c r="I24">
-        <v>-1.83517460215112</v>
+        <v>-4.34069631336406</v>
       </c>
       <c r="J24">
-        <v>0.0066993300669933</v>
+        <v>0.0014998500149985</v>
       </c>
       <c r="K24">
-        <v>0.0233119545188338</v>
+        <v>0.008443600084436001</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -1316,28 +1319,28 @@
         <v>23</v>
       </c>
       <c r="D25">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E25">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F25">
-        <v>-0.0599898743143231</v>
+        <v>-0.123628811696748</v>
       </c>
       <c r="G25">
-        <v>-8.191505173600831</v>
+        <v>-14.8039028862857</v>
       </c>
       <c r="H25">
-        <v>-14.5411634089298</v>
+        <v>-23.8710768148773</v>
       </c>
       <c r="I25">
-        <v>-1.49104851089367</v>
+        <v>-6.35959789070967</v>
       </c>
       <c r="J25">
-        <v>0.0121987801219878</v>
+        <v>0.0018998100189981</v>
       </c>
       <c r="K25">
-        <v>0.0330633603306336</v>
+        <v>0.008443600084436001</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -1351,28 +1354,28 @@
         <v>24</v>
       </c>
       <c r="D26">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E26">
-        <v>40</v>
+        <v>160</v>
       </c>
       <c r="F26">
-        <v>-0.00304831497652741</v>
+        <v>-0.00142513905768987</v>
       </c>
       <c r="G26">
-        <v>-9.672578209827989</v>
+        <v>-3.90327732690893</v>
       </c>
       <c r="H26">
-        <v>-20.5697924579183</v>
+        <v>-7.73803690498597</v>
       </c>
       <c r="I26">
-        <v>2.67417161860893</v>
+        <v>0.00775858920047114</v>
       </c>
       <c r="J26">
-        <v>0.0724927507249275</v>
+        <v>0.0296970302969703</v>
       </c>
       <c r="K26">
-        <v>0.108739126087391</v>
+        <v>0.04242432899567185</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -1386,28 +1389,28 @@
         <v>24</v>
       </c>
       <c r="D27">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E27">
-        <v>40</v>
+        <v>160</v>
       </c>
       <c r="F27">
-        <v>-0.00352077842517948</v>
+        <v>-0.00200997216469339</v>
       </c>
       <c r="G27">
-        <v>-11.3554591278585</v>
+        <v>-5.44671551832906</v>
       </c>
       <c r="H27">
-        <v>-23.7274162042636</v>
+        <v>-9.564714776353799</v>
       </c>
       <c r="I27">
-        <v>3.22641189793946</v>
+        <v>-1.34184929226255</v>
       </c>
       <c r="J27">
-        <v>0.0656934306569343</v>
+        <v>0.0054994500549945</v>
       </c>
       <c r="K27">
-        <v>0.101610092155341</v>
+        <v>0.01571271444284143</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -1421,28 +1424,28 @@
         <v>24</v>
       </c>
       <c r="D28">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E28">
-        <v>40</v>
+        <v>160</v>
       </c>
       <c r="F28">
-        <v>-0.695899274342389</v>
+        <v>-0.38718347675304</v>
       </c>
       <c r="G28">
-        <v>-12.0137367090493</v>
+        <v>-6.70973371481666</v>
       </c>
       <c r="H28">
-        <v>-29.5182254753519</v>
+        <v>-12.8480119771694</v>
       </c>
       <c r="I28">
-        <v>4.93347873373744</v>
+        <v>-0.681260034655301</v>
       </c>
       <c r="J28">
-        <v>0.111188881111889</v>
+        <v>0.0194980501949805</v>
       </c>
       <c r="K28">
-        <v>0.146754555313699</v>
+        <v>0.03390965251300956</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -1456,28 +1459,28 @@
         <v>24</v>
       </c>
       <c r="D29">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E29">
-        <v>40</v>
+        <v>160</v>
       </c>
       <c r="F29">
-        <v>-0.617605006371476</v>
+        <v>-0.485112114343369</v>
       </c>
       <c r="G29">
-        <v>-11.1297925131819</v>
+        <v>-8.342471246999761</v>
       </c>
       <c r="H29">
-        <v>-28.0249564442272</v>
+        <v>-14.1889752040962</v>
       </c>
       <c r="I29">
-        <v>8.085464884682629</v>
+        <v>-2.55205053892857</v>
       </c>
       <c r="J29">
-        <v>0.13988601139886</v>
+        <v>0.0047995200479952</v>
       </c>
       <c r="K29">
-        <v>0.168703129687031</v>
+        <v>0.01476775399383139</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -1491,28 +1494,28 @@
         <v>24</v>
       </c>
       <c r="D30">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E30">
-        <v>40</v>
+        <v>160</v>
       </c>
       <c r="F30">
-        <v>-1.15942235886815</v>
+        <v>-0.41223661230812</v>
       </c>
       <c r="G30">
-        <v>-31.5553369534262</v>
+        <v>-12.5494977568365</v>
       </c>
       <c r="H30">
-        <v>-43.2337172629337</v>
+        <v>-20.0549353616032</v>
       </c>
       <c r="I30">
-        <v>-16.007443948737</v>
+        <v>-4.86520404681452</v>
       </c>
       <c r="J30">
-        <v>0.0028997100289971</v>
+        <v>0.0016998300169983</v>
       </c>
       <c r="K30">
-        <v>0.0156506088521583</v>
+        <v>0.008443600084436001</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -1526,28 +1529,28 @@
         <v>24</v>
       </c>
       <c r="D31">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E31">
-        <v>40</v>
+        <v>160</v>
       </c>
       <c r="F31">
-        <v>-1.03198600944061</v>
+        <v>-0.377330413617452</v>
       </c>
       <c r="G31">
-        <v>-29.1547827812484</v>
+        <v>-11.6114789432087</v>
       </c>
       <c r="H31">
-        <v>-42.9348631518719</v>
+        <v>-19.7712949536142</v>
       </c>
       <c r="I31">
-        <v>-8.648506123125051</v>
+        <v>-2.7325181737937</v>
       </c>
       <c r="J31">
-        <v>0.0156984301569843</v>
+        <v>0.0074992500749925</v>
       </c>
       <c r="K31">
-        <v>0.0384451350783289</v>
+        <v>0.01874812518748125</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -1561,28 +1564,28 @@
         <v>24</v>
       </c>
       <c r="D32">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E32">
-        <v>40</v>
+        <v>160</v>
       </c>
       <c r="F32">
-        <v>-0.13270094153788</v>
+        <v>-0.0531821350745159</v>
       </c>
       <c r="G32">
-        <v>-16.9285432750099</v>
+        <v>-7.19617057069742</v>
       </c>
       <c r="H32">
-        <v>-25.1902736148939</v>
+        <v>-12.2095432994123</v>
       </c>
       <c r="I32">
-        <v>-5.06047395886088</v>
+        <v>-1.83517460215112</v>
       </c>
       <c r="J32">
-        <v>0.0137986201379862</v>
+        <v>0.0066993300669933</v>
       </c>
       <c r="K32">
-        <v>0.035996400359964</v>
+        <v>0.0178648801786488</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -1596,28 +1599,308 @@
         <v>24</v>
       </c>
       <c r="D33">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="E33">
+        <v>160</v>
+      </c>
+      <c r="F33">
+        <v>-0.0599898743143231</v>
+      </c>
+      <c r="G33">
+        <v>-8.191505173600831</v>
+      </c>
+      <c r="H33">
+        <v>-14.5411634089298</v>
+      </c>
+      <c r="I33">
+        <v>-1.49104851089367</v>
+      </c>
+      <c r="J33">
+        <v>0.0121987801219878</v>
+      </c>
+      <c r="K33">
+        <v>0.0243975602439756</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
+      <c r="A34" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D34">
+        <v>22</v>
+      </c>
+      <c r="E34">
         <v>40</v>
       </c>
-      <c r="F33">
+      <c r="F34">
+        <v>-0.00304831497652741</v>
+      </c>
+      <c r="G34">
+        <v>-9.672578209827989</v>
+      </c>
+      <c r="H34">
+        <v>-20.5697924579183</v>
+      </c>
+      <c r="I34">
+        <v>2.67417161860893</v>
+      </c>
+      <c r="J34">
+        <v>0.0724927507249275</v>
+      </c>
+      <c r="K34">
+        <v>0.09061593840615938</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11">
+      <c r="A35" t="s">
+        <v>15</v>
+      </c>
+      <c r="B35" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35">
+        <v>22</v>
+      </c>
+      <c r="E35">
+        <v>40</v>
+      </c>
+      <c r="F35">
+        <v>-0.00352077842517948</v>
+      </c>
+      <c r="G35">
+        <v>-11.3554591278585</v>
+      </c>
+      <c r="H35">
+        <v>-23.7274162042636</v>
+      </c>
+      <c r="I35">
+        <v>3.22641189793946</v>
+      </c>
+      <c r="J35">
+        <v>0.0656934306569343</v>
+      </c>
+      <c r="K35">
+        <v>0.08476571697668941</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11">
+      <c r="A36" t="s">
+        <v>19</v>
+      </c>
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" t="s">
+        <v>25</v>
+      </c>
+      <c r="D36">
+        <v>22</v>
+      </c>
+      <c r="E36">
+        <v>40</v>
+      </c>
+      <c r="F36">
+        <v>-0.695899274342389</v>
+      </c>
+      <c r="G36">
+        <v>-12.0137367090493</v>
+      </c>
+      <c r="H36">
+        <v>-29.5182254753519</v>
+      </c>
+      <c r="I36">
+        <v>4.93347873373744</v>
+      </c>
+      <c r="J36">
+        <v>0.111188881111889</v>
+      </c>
+      <c r="K36">
+        <v>0.1235432012354322</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
+      <c r="A37" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37">
+        <v>22</v>
+      </c>
+      <c r="E37">
+        <v>40</v>
+      </c>
+      <c r="F37">
+        <v>-0.617605006371476</v>
+      </c>
+      <c r="G37">
+        <v>-11.1297925131819</v>
+      </c>
+      <c r="H37">
+        <v>-28.0249564442272</v>
+      </c>
+      <c r="I37">
+        <v>8.085464884682629</v>
+      </c>
+      <c r="J37">
+        <v>0.13988601139886</v>
+      </c>
+      <c r="K37">
+        <v>0.143472832203959</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
+      <c r="A38" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" t="s">
+        <v>25</v>
+      </c>
+      <c r="D38">
+        <v>22</v>
+      </c>
+      <c r="E38">
+        <v>40</v>
+      </c>
+      <c r="F38">
+        <v>-1.15942235886815</v>
+      </c>
+      <c r="G38">
+        <v>-31.5553369534262</v>
+      </c>
+      <c r="H38">
+        <v>-43.2337172629337</v>
+      </c>
+      <c r="I38">
+        <v>-16.007443948737</v>
+      </c>
+      <c r="J38">
+        <v>0.0028997100289971</v>
+      </c>
+      <c r="K38">
+        <v>0.01090800010908</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
+      <c r="A39" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D39">
+        <v>22</v>
+      </c>
+      <c r="E39">
+        <v>40</v>
+      </c>
+      <c r="F39">
+        <v>-1.03198600944061</v>
+      </c>
+      <c r="G39">
+        <v>-29.1547827812484</v>
+      </c>
+      <c r="H39">
+        <v>-42.9348631518719</v>
+      </c>
+      <c r="I39">
+        <v>-8.648506123125051</v>
+      </c>
+      <c r="J39">
+        <v>0.0156984301569843</v>
+      </c>
+      <c r="K39">
+        <v>0.028542600285426</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
+      <c r="A40" t="s">
+        <v>21</v>
+      </c>
+      <c r="B40" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" t="s">
+        <v>25</v>
+      </c>
+      <c r="D40">
+        <v>22</v>
+      </c>
+      <c r="E40">
+        <v>40</v>
+      </c>
+      <c r="F40">
+        <v>-0.13270094153788</v>
+      </c>
+      <c r="G40">
+        <v>-16.9285432750099</v>
+      </c>
+      <c r="H40">
+        <v>-25.1902736148939</v>
+      </c>
+      <c r="I40">
+        <v>-5.06047395886088</v>
+      </c>
+      <c r="J40">
+        <v>0.0137986201379862</v>
+      </c>
+      <c r="K40">
+        <v>0.02628308597711657</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41" t="s">
+        <v>21</v>
+      </c>
+      <c r="B41" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" t="s">
+        <v>25</v>
+      </c>
+      <c r="D41">
+        <v>22</v>
+      </c>
+      <c r="E41">
+        <v>40</v>
+      </c>
+      <c r="F41">
         <v>-0.167890570878149</v>
       </c>
-      <c r="G33">
+      <c r="G41">
         <v>-21.7667058326155</v>
       </c>
-      <c r="H33">
+      <c r="H41">
         <v>-34.4501620574432</v>
       </c>
-      <c r="I33">
+      <c r="I41">
         <v>-8.15156886464333</v>
       </c>
-      <c r="J33">
+      <c r="J41">
         <v>0.009899010098990101</v>
       </c>
-      <c r="K33">
-        <v>0.0282828859971146</v>
+      <c r="K41">
+        <v>0.021997800219978</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Table 2: Mid+High and High sites columns removed (all site-years + the two years-with-mortality columns, as Fig 2b; stars unchanged); copy_to_coauthor_draft.sh kept in the project; seeded jitter in 51; package source data updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flux/paper_code_data/source_data/Table2_siteyear_MAE_bootstrap.xlsx
+++ b/data/flux/paper_code_data/source_data/Table2_siteyear_MAE_bootstrap.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="24">
   <si>
     <t>note</t>
   </si>
@@ -26,7 +26,7 @@
     <t>pct = % change; pct_lo/pct_hi = 95 % site-block bootstrap interval; p_perm/q = paired permutation (sites swapped), BH-corrected across the AutoGluon site-year tests.</t>
   </si>
   <si>
-    <t>subset: all = all site-years; midhigh / high = all years of the Mid+High / High sites; yr_midhigh / yr_high = site-years whose own relative mortality exceeds the Mid / High break.</t>
+    <t>subset: all = all site-years; yr_midhigh / yr_high = site-years whose own relative mortality exceeds the Mid (10.6 %) / High (24.0 %) break; q corrected over all AutoGluon site-year tests, as in the draft.</t>
   </si>
   <si>
     <t>response</t>
@@ -81,12 +81,6 @@
   </si>
   <si>
     <t>WUE</t>
-  </si>
-  <si>
-    <t>midhigh</t>
-  </si>
-  <si>
-    <t>high</t>
   </si>
   <si>
     <t>yr_midhigh</t>
@@ -465,7 +459,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1">
@@ -797,25 +791,25 @@
         <v>60</v>
       </c>
       <c r="E10">
-        <v>225</v>
+        <v>160</v>
       </c>
       <c r="F10">
-        <v>-0.0007707274229183521</v>
+        <v>-0.00142513905768987</v>
       </c>
       <c r="G10">
-        <v>-2.06028814037544</v>
+        <v>-3.90327732690893</v>
       </c>
       <c r="H10">
-        <v>-5.25039418056846</v>
+        <v>-7.73803690498597</v>
       </c>
       <c r="I10">
-        <v>1.09525253577241</v>
+        <v>0.00775858920047114</v>
       </c>
       <c r="J10">
-        <v>0.103689631036896</v>
+        <v>0.0296970302969703</v>
       </c>
       <c r="K10">
-        <v>0.1219878012198777</v>
+        <v>0.04242432899567185</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -832,25 +826,25 @@
         <v>60</v>
       </c>
       <c r="E11">
-        <v>225</v>
+        <v>160</v>
       </c>
       <c r="F11">
-        <v>-0.00139125428838921</v>
+        <v>-0.00200997216469339</v>
       </c>
       <c r="G11">
-        <v>-3.69334130316401</v>
+        <v>-5.44671551832906</v>
       </c>
       <c r="H11">
-        <v>-7.25499787567919</v>
+        <v>-9.564714776353799</v>
       </c>
       <c r="I11">
-        <v>-0.071805817701489</v>
+        <v>-1.34184929226255</v>
       </c>
       <c r="J11">
-        <v>0.023997600239976</v>
+        <v>0.0054994500549945</v>
       </c>
       <c r="K11">
-        <v>0.03555200035552</v>
+        <v>0.01571271444284143</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -867,25 +861,25 @@
         <v>60</v>
       </c>
       <c r="E12">
-        <v>225</v>
+        <v>160</v>
       </c>
       <c r="F12">
-        <v>-0.35150318006165</v>
+        <v>-0.38718347675304</v>
       </c>
       <c r="G12">
-        <v>-6.12976587101762</v>
+        <v>-6.70973371481666</v>
       </c>
       <c r="H12">
-        <v>-10.9151964237536</v>
+        <v>-12.8480119771694</v>
       </c>
       <c r="I12">
-        <v>-1.46265082042202</v>
+        <v>-0.681260034655301</v>
       </c>
       <c r="J12">
-        <v>0.009099090090990899</v>
+        <v>0.0194980501949805</v>
       </c>
       <c r="K12">
-        <v>0.021409623743508</v>
+        <v>0.03390965251300956</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -902,25 +896,25 @@
         <v>60</v>
       </c>
       <c r="E13">
-        <v>225</v>
+        <v>160</v>
       </c>
       <c r="F13">
-        <v>-0.485195323601988</v>
+        <v>-0.485112114343369</v>
       </c>
       <c r="G13">
-        <v>-8.28300520124635</v>
+        <v>-8.342471246999761</v>
       </c>
       <c r="H13">
-        <v>-12.6023981414942</v>
+        <v>-14.1889752040962</v>
       </c>
       <c r="I13">
-        <v>-3.98249083629758</v>
+        <v>-2.55205053892857</v>
       </c>
       <c r="J13">
-        <v>0.0007999200079992</v>
+        <v>0.0047995200479952</v>
       </c>
       <c r="K13">
-        <v>0.0063993600639936</v>
+        <v>0.01476775399383139</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -937,25 +931,25 @@
         <v>60</v>
       </c>
       <c r="E14">
-        <v>225</v>
+        <v>160</v>
       </c>
       <c r="F14">
-        <v>-0.351166347256085</v>
+        <v>-0.41223661230812</v>
       </c>
       <c r="G14">
-        <v>-11.3168217363717</v>
+        <v>-12.5494977568365</v>
       </c>
       <c r="H14">
-        <v>-17.481015644899</v>
+        <v>-20.0549353616032</v>
       </c>
       <c r="I14">
-        <v>-5.08037980606321</v>
+        <v>-4.86520404681452</v>
       </c>
       <c r="J14">
-        <v>0.0003999600039996</v>
+        <v>0.0016998300169983</v>
       </c>
       <c r="K14">
-        <v>0.005332800053328</v>
+        <v>0.008443600084436001</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -972,25 +966,25 @@
         <v>60</v>
       </c>
       <c r="E15">
-        <v>225</v>
+        <v>160</v>
       </c>
       <c r="F15">
-        <v>-0.327016264315909</v>
+        <v>-0.377330413617452</v>
       </c>
       <c r="G15">
-        <v>-10.5302835080963</v>
+        <v>-11.6114789432087</v>
       </c>
       <c r="H15">
-        <v>-17.3196912634385</v>
+        <v>-19.7712949536142</v>
       </c>
       <c r="I15">
-        <v>-3.39598341143336</v>
+        <v>-2.7325181737937</v>
       </c>
       <c r="J15">
-        <v>0.0045995400459954</v>
+        <v>0.0074992500749925</v>
       </c>
       <c r="K15">
-        <v>0.01476775399383139</v>
+        <v>0.01874812518748125</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1007,25 +1001,25 @@
         <v>60</v>
       </c>
       <c r="E16">
-        <v>225</v>
+        <v>160</v>
       </c>
       <c r="F16">
-        <v>-0.0489410796311922</v>
+        <v>-0.0531821350745159</v>
       </c>
       <c r="G16">
-        <v>-6.84773054808714</v>
+        <v>-7.19617057069742</v>
       </c>
       <c r="H16">
-        <v>-11.2744963976347</v>
+        <v>-12.2095432994123</v>
       </c>
       <c r="I16">
-        <v>-2.31010483748635</v>
+        <v>-1.83517460215112</v>
       </c>
       <c r="J16">
-        <v>0.0016998300169983</v>
+        <v>0.0066993300669933</v>
       </c>
       <c r="K16">
-        <v>0.008443600084436001</v>
+        <v>0.0178648801786488</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1042,22 +1036,22 @@
         <v>60</v>
       </c>
       <c r="E17">
-        <v>225</v>
+        <v>160</v>
       </c>
       <c r="F17">
-        <v>-0.0450009480014665</v>
+        <v>-0.0599898743143231</v>
       </c>
       <c r="G17">
-        <v>-6.4011798237569</v>
+        <v>-8.191505173600831</v>
       </c>
       <c r="H17">
-        <v>-11.5077326742567</v>
+        <v>-14.5411634089298</v>
       </c>
       <c r="I17">
-        <v>-1.1650061934816</v>
+        <v>-1.49104851089367</v>
       </c>
       <c r="J17">
-        <v>0.0116988301169883</v>
+        <v>0.0121987801219878</v>
       </c>
       <c r="K17">
         <v>0.0243975602439756</v>
@@ -1077,25 +1071,25 @@
         <v>22</v>
       </c>
       <c r="E18">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F18">
-        <v>-0.00122773386165283</v>
+        <v>-0.00304831497652741</v>
       </c>
       <c r="G18">
-        <v>-2.94197075180864</v>
+        <v>-9.672578209827989</v>
       </c>
       <c r="H18">
-        <v>-8.375869844590399</v>
+        <v>-20.5697924579183</v>
       </c>
       <c r="I18">
-        <v>2.13138272699604</v>
+        <v>2.67417161860893</v>
       </c>
       <c r="J18">
-        <v>0.128287171282872</v>
+        <v>0.0724927507249275</v>
       </c>
       <c r="K18">
-        <v>0.1350391276661811</v>
+        <v>0.09061593840615938</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -1112,25 +1106,25 @@
         <v>22</v>
       </c>
       <c r="E19">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F19">
-        <v>-0.00218117436495249</v>
+        <v>-0.00352077842517948</v>
       </c>
       <c r="G19">
-        <v>-5.25048299349444</v>
+        <v>-11.3554591278585</v>
       </c>
       <c r="H19">
-        <v>-13.1430006443466</v>
+        <v>-23.7274162042636</v>
       </c>
       <c r="I19">
-        <v>1.24909337767268</v>
+        <v>3.22641189793946</v>
       </c>
       <c r="J19">
-        <v>0.0591940805919408</v>
+        <v>0.0656934306569343</v>
       </c>
       <c r="K19">
-        <v>0.0789254407892544</v>
+        <v>0.08476571697668941</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -1147,22 +1141,22 @@
         <v>22</v>
       </c>
       <c r="E20">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F20">
-        <v>-0.407422486981712</v>
+        <v>-0.695899274342389</v>
       </c>
       <c r="G20">
-        <v>-7.19093289074554</v>
+        <v>-12.0137367090493</v>
       </c>
       <c r="H20">
-        <v>-18.0528336887189</v>
+        <v>-29.5182254753519</v>
       </c>
       <c r="I20">
-        <v>2.87646398667019</v>
+        <v>4.93347873373744</v>
       </c>
       <c r="J20">
-        <v>0.108889111088891</v>
+        <v>0.111188881111889</v>
       </c>
       <c r="K20">
         <v>0.1235432012354322</v>
@@ -1182,25 +1176,25 @@
         <v>22</v>
       </c>
       <c r="E21">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F21">
-        <v>-0.386929315382964</v>
+        <v>-0.617605006371476</v>
       </c>
       <c r="G21">
-        <v>-7.0535023162857</v>
+        <v>-11.1297925131819</v>
       </c>
       <c r="H21">
-        <v>-17.2276326820933</v>
+        <v>-28.0249564442272</v>
       </c>
       <c r="I21">
-        <v>3.60442454025906</v>
+        <v>8.085464884682629</v>
       </c>
       <c r="J21">
-        <v>0.118688131186881</v>
+        <v>0.13988601139886</v>
       </c>
       <c r="K21">
-        <v>0.1283114931750065</v>
+        <v>0.143472832203959</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1217,25 +1211,25 @@
         <v>22</v>
       </c>
       <c r="E22">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F22">
-        <v>-0.691097880501684</v>
+        <v>-1.15942235886815</v>
       </c>
       <c r="G22">
-        <v>-22.6321346731244</v>
+        <v>-31.5553369534262</v>
       </c>
       <c r="H22">
-        <v>-33.5912532572929</v>
+        <v>-43.2337172629337</v>
       </c>
       <c r="I22">
-        <v>-11.0593782395689</v>
+        <v>-16.007443948737</v>
       </c>
       <c r="J22">
-        <v>0.0007999200079992</v>
+        <v>0.0028997100289971</v>
       </c>
       <c r="K22">
-        <v>0.0063993600639936</v>
+        <v>0.01090800010908</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -1252,25 +1246,25 @@
         <v>22</v>
       </c>
       <c r="E23">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F23">
-        <v>-0.499947499305979</v>
+        <v>-1.03198600944061</v>
       </c>
       <c r="G23">
-        <v>-17.4786290491947</v>
+        <v>-29.1547827812484</v>
       </c>
       <c r="H23">
-        <v>-30.6844457896897</v>
+        <v>-42.9348631518719</v>
       </c>
       <c r="I23">
-        <v>-2.09408633866107</v>
+        <v>-8.648506123125051</v>
       </c>
       <c r="J23">
-        <v>0.0311968803119688</v>
+        <v>0.0156984301569843</v>
       </c>
       <c r="K23">
-        <v>0.04303017974064662</v>
+        <v>0.028542600285426</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -1287,25 +1281,25 @@
         <v>22</v>
       </c>
       <c r="E24">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F24">
-        <v>-0.0919717941041224</v>
+        <v>-0.13270094153788</v>
       </c>
       <c r="G24">
-        <v>-10.9330213731233</v>
+        <v>-16.9285432750099</v>
       </c>
       <c r="H24">
-        <v>-17.7875005238154</v>
+        <v>-25.1902736148939</v>
       </c>
       <c r="I24">
-        <v>-4.34069631336406</v>
+        <v>-5.06047395886088</v>
       </c>
       <c r="J24">
-        <v>0.0014998500149985</v>
+        <v>0.0137986201379862</v>
       </c>
       <c r="K24">
-        <v>0.008443600084436001</v>
+        <v>0.02628308597711657</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -1322,584 +1316,24 @@
         <v>22</v>
       </c>
       <c r="E25">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F25">
-        <v>-0.123628811696748</v>
+        <v>-0.167890570878149</v>
       </c>
       <c r="G25">
-        <v>-14.8039028862857</v>
+        <v>-21.7667058326155</v>
       </c>
       <c r="H25">
-        <v>-23.8710768148773</v>
+        <v>-34.4501620574432</v>
       </c>
       <c r="I25">
-        <v>-6.35959789070967</v>
+        <v>-8.15156886464333</v>
       </c>
       <c r="J25">
-        <v>0.0018998100189981</v>
+        <v>0.009899010098990101</v>
       </c>
       <c r="K25">
-        <v>0.008443600084436001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
-      <c r="A26" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" t="s">
-        <v>24</v>
-      </c>
-      <c r="D26">
-        <v>60</v>
-      </c>
-      <c r="E26">
-        <v>160</v>
-      </c>
-      <c r="F26">
-        <v>-0.00142513905768987</v>
-      </c>
-      <c r="G26">
-        <v>-3.90327732690893</v>
-      </c>
-      <c r="H26">
-        <v>-7.73803690498597</v>
-      </c>
-      <c r="I26">
-        <v>0.00775858920047114</v>
-      </c>
-      <c r="J26">
-        <v>0.0296970302969703</v>
-      </c>
-      <c r="K26">
-        <v>0.04242432899567185</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="A27" t="s">
-        <v>15</v>
-      </c>
-      <c r="B27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" t="s">
-        <v>24</v>
-      </c>
-      <c r="D27">
-        <v>60</v>
-      </c>
-      <c r="E27">
-        <v>160</v>
-      </c>
-      <c r="F27">
-        <v>-0.00200997216469339</v>
-      </c>
-      <c r="G27">
-        <v>-5.44671551832906</v>
-      </c>
-      <c r="H27">
-        <v>-9.564714776353799</v>
-      </c>
-      <c r="I27">
-        <v>-1.34184929226255</v>
-      </c>
-      <c r="J27">
-        <v>0.0054994500549945</v>
-      </c>
-      <c r="K27">
-        <v>0.01571271444284143</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="A28" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" t="s">
-        <v>16</v>
-      </c>
-      <c r="C28" t="s">
-        <v>24</v>
-      </c>
-      <c r="D28">
-        <v>60</v>
-      </c>
-      <c r="E28">
-        <v>160</v>
-      </c>
-      <c r="F28">
-        <v>-0.38718347675304</v>
-      </c>
-      <c r="G28">
-        <v>-6.70973371481666</v>
-      </c>
-      <c r="H28">
-        <v>-12.8480119771694</v>
-      </c>
-      <c r="I28">
-        <v>-0.681260034655301</v>
-      </c>
-      <c r="J28">
-        <v>0.0194980501949805</v>
-      </c>
-      <c r="K28">
-        <v>0.03390965251300956</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="A29" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" t="s">
-        <v>18</v>
-      </c>
-      <c r="C29" t="s">
-        <v>24</v>
-      </c>
-      <c r="D29">
-        <v>60</v>
-      </c>
-      <c r="E29">
-        <v>160</v>
-      </c>
-      <c r="F29">
-        <v>-0.485112114343369</v>
-      </c>
-      <c r="G29">
-        <v>-8.342471246999761</v>
-      </c>
-      <c r="H29">
-        <v>-14.1889752040962</v>
-      </c>
-      <c r="I29">
-        <v>-2.55205053892857</v>
-      </c>
-      <c r="J29">
-        <v>0.0047995200479952</v>
-      </c>
-      <c r="K29">
-        <v>0.01476775399383139</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
-      <c r="A30" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" t="s">
-        <v>24</v>
-      </c>
-      <c r="D30">
-        <v>60</v>
-      </c>
-      <c r="E30">
-        <v>160</v>
-      </c>
-      <c r="F30">
-        <v>-0.41223661230812</v>
-      </c>
-      <c r="G30">
-        <v>-12.5494977568365</v>
-      </c>
-      <c r="H30">
-        <v>-20.0549353616032</v>
-      </c>
-      <c r="I30">
-        <v>-4.86520404681452</v>
-      </c>
-      <c r="J30">
-        <v>0.0016998300169983</v>
-      </c>
-      <c r="K30">
-        <v>0.008443600084436001</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
-      <c r="A31" t="s">
-        <v>20</v>
-      </c>
-      <c r="B31" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" t="s">
-        <v>24</v>
-      </c>
-      <c r="D31">
-        <v>60</v>
-      </c>
-      <c r="E31">
-        <v>160</v>
-      </c>
-      <c r="F31">
-        <v>-0.377330413617452</v>
-      </c>
-      <c r="G31">
-        <v>-11.6114789432087</v>
-      </c>
-      <c r="H31">
-        <v>-19.7712949536142</v>
-      </c>
-      <c r="I31">
-        <v>-2.7325181737937</v>
-      </c>
-      <c r="J31">
-        <v>0.0074992500749925</v>
-      </c>
-      <c r="K31">
-        <v>0.01874812518748125</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
-      <c r="A32" t="s">
-        <v>21</v>
-      </c>
-      <c r="B32" t="s">
-        <v>16</v>
-      </c>
-      <c r="C32" t="s">
-        <v>24</v>
-      </c>
-      <c r="D32">
-        <v>60</v>
-      </c>
-      <c r="E32">
-        <v>160</v>
-      </c>
-      <c r="F32">
-        <v>-0.0531821350745159</v>
-      </c>
-      <c r="G32">
-        <v>-7.19617057069742</v>
-      </c>
-      <c r="H32">
-        <v>-12.2095432994123</v>
-      </c>
-      <c r="I32">
-        <v>-1.83517460215112</v>
-      </c>
-      <c r="J32">
-        <v>0.0066993300669933</v>
-      </c>
-      <c r="K32">
-        <v>0.0178648801786488</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11">
-      <c r="A33" t="s">
-        <v>21</v>
-      </c>
-      <c r="B33" t="s">
-        <v>18</v>
-      </c>
-      <c r="C33" t="s">
-        <v>24</v>
-      </c>
-      <c r="D33">
-        <v>60</v>
-      </c>
-      <c r="E33">
-        <v>160</v>
-      </c>
-      <c r="F33">
-        <v>-0.0599898743143231</v>
-      </c>
-      <c r="G33">
-        <v>-8.191505173600831</v>
-      </c>
-      <c r="H33">
-        <v>-14.5411634089298</v>
-      </c>
-      <c r="I33">
-        <v>-1.49104851089367</v>
-      </c>
-      <c r="J33">
-        <v>0.0121987801219878</v>
-      </c>
-      <c r="K33">
-        <v>0.0243975602439756</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11">
-      <c r="A34" t="s">
-        <v>15</v>
-      </c>
-      <c r="B34" t="s">
-        <v>16</v>
-      </c>
-      <c r="C34" t="s">
-        <v>25</v>
-      </c>
-      <c r="D34">
-        <v>22</v>
-      </c>
-      <c r="E34">
-        <v>40</v>
-      </c>
-      <c r="F34">
-        <v>-0.00304831497652741</v>
-      </c>
-      <c r="G34">
-        <v>-9.672578209827989</v>
-      </c>
-      <c r="H34">
-        <v>-20.5697924579183</v>
-      </c>
-      <c r="I34">
-        <v>2.67417161860893</v>
-      </c>
-      <c r="J34">
-        <v>0.0724927507249275</v>
-      </c>
-      <c r="K34">
-        <v>0.09061593840615938</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11">
-      <c r="A35" t="s">
-        <v>15</v>
-      </c>
-      <c r="B35" t="s">
-        <v>18</v>
-      </c>
-      <c r="C35" t="s">
-        <v>25</v>
-      </c>
-      <c r="D35">
-        <v>22</v>
-      </c>
-      <c r="E35">
-        <v>40</v>
-      </c>
-      <c r="F35">
-        <v>-0.00352077842517948</v>
-      </c>
-      <c r="G35">
-        <v>-11.3554591278585</v>
-      </c>
-      <c r="H35">
-        <v>-23.7274162042636</v>
-      </c>
-      <c r="I35">
-        <v>3.22641189793946</v>
-      </c>
-      <c r="J35">
-        <v>0.0656934306569343</v>
-      </c>
-      <c r="K35">
-        <v>0.08476571697668941</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11">
-      <c r="A36" t="s">
-        <v>19</v>
-      </c>
-      <c r="B36" t="s">
-        <v>16</v>
-      </c>
-      <c r="C36" t="s">
-        <v>25</v>
-      </c>
-      <c r="D36">
-        <v>22</v>
-      </c>
-      <c r="E36">
-        <v>40</v>
-      </c>
-      <c r="F36">
-        <v>-0.695899274342389</v>
-      </c>
-      <c r="G36">
-        <v>-12.0137367090493</v>
-      </c>
-      <c r="H36">
-        <v>-29.5182254753519</v>
-      </c>
-      <c r="I36">
-        <v>4.93347873373744</v>
-      </c>
-      <c r="J36">
-        <v>0.111188881111889</v>
-      </c>
-      <c r="K36">
-        <v>0.1235432012354322</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11">
-      <c r="A37" t="s">
-        <v>19</v>
-      </c>
-      <c r="B37" t="s">
-        <v>18</v>
-      </c>
-      <c r="C37" t="s">
-        <v>25</v>
-      </c>
-      <c r="D37">
-        <v>22</v>
-      </c>
-      <c r="E37">
-        <v>40</v>
-      </c>
-      <c r="F37">
-        <v>-0.617605006371476</v>
-      </c>
-      <c r="G37">
-        <v>-11.1297925131819</v>
-      </c>
-      <c r="H37">
-        <v>-28.0249564442272</v>
-      </c>
-      <c r="I37">
-        <v>8.085464884682629</v>
-      </c>
-      <c r="J37">
-        <v>0.13988601139886</v>
-      </c>
-      <c r="K37">
-        <v>0.143472832203959</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11">
-      <c r="A38" t="s">
-        <v>20</v>
-      </c>
-      <c r="B38" t="s">
-        <v>16</v>
-      </c>
-      <c r="C38" t="s">
-        <v>25</v>
-      </c>
-      <c r="D38">
-        <v>22</v>
-      </c>
-      <c r="E38">
-        <v>40</v>
-      </c>
-      <c r="F38">
-        <v>-1.15942235886815</v>
-      </c>
-      <c r="G38">
-        <v>-31.5553369534262</v>
-      </c>
-      <c r="H38">
-        <v>-43.2337172629337</v>
-      </c>
-      <c r="I38">
-        <v>-16.007443948737</v>
-      </c>
-      <c r="J38">
-        <v>0.0028997100289971</v>
-      </c>
-      <c r="K38">
-        <v>0.01090800010908</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11">
-      <c r="A39" t="s">
-        <v>20</v>
-      </c>
-      <c r="B39" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39" t="s">
-        <v>25</v>
-      </c>
-      <c r="D39">
-        <v>22</v>
-      </c>
-      <c r="E39">
-        <v>40</v>
-      </c>
-      <c r="F39">
-        <v>-1.03198600944061</v>
-      </c>
-      <c r="G39">
-        <v>-29.1547827812484</v>
-      </c>
-      <c r="H39">
-        <v>-42.9348631518719</v>
-      </c>
-      <c r="I39">
-        <v>-8.648506123125051</v>
-      </c>
-      <c r="J39">
-        <v>0.0156984301569843</v>
-      </c>
-      <c r="K39">
-        <v>0.028542600285426</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11">
-      <c r="A40" t="s">
-        <v>21</v>
-      </c>
-      <c r="B40" t="s">
-        <v>16</v>
-      </c>
-      <c r="C40" t="s">
-        <v>25</v>
-      </c>
-      <c r="D40">
-        <v>22</v>
-      </c>
-      <c r="E40">
-        <v>40</v>
-      </c>
-      <c r="F40">
-        <v>-0.13270094153788</v>
-      </c>
-      <c r="G40">
-        <v>-16.9285432750099</v>
-      </c>
-      <c r="H40">
-        <v>-25.1902736148939</v>
-      </c>
-      <c r="I40">
-        <v>-5.06047395886088</v>
-      </c>
-      <c r="J40">
-        <v>0.0137986201379862</v>
-      </c>
-      <c r="K40">
-        <v>0.02628308597711657</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11">
-      <c r="A41" t="s">
-        <v>21</v>
-      </c>
-      <c r="B41" t="s">
-        <v>18</v>
-      </c>
-      <c r="C41" t="s">
-        <v>25</v>
-      </c>
-      <c r="D41">
-        <v>22</v>
-      </c>
-      <c r="E41">
-        <v>40</v>
-      </c>
-      <c r="F41">
-        <v>-0.167890570878149</v>
-      </c>
-      <c r="G41">
-        <v>-21.7667058326155</v>
-      </c>
-      <c r="H41">
-        <v>-34.4501620574432</v>
-      </c>
-      <c r="I41">
-        <v>-8.15156886464333</v>
-      </c>
-      <c r="J41">
-        <v>0.009899010098990101</v>
-      </c>
-      <c r="K41">
         <v>0.021997800219978</v>
       </c>
     </row>

</xml_diff>